<commit_message>
fix: normalização insensível a maiúsculas/minúsculas para pareamento de obras (Hall Design vs HALL DESIGN) e consolidação total de lançamentos manuais
</commit_message>
<xml_diff>
--- a/INFORMAÇÕES_PROJETOS.xlsx
+++ b/INFORMAÇÕES_PROJETOS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HomePC\.gemini\antigravity-ide\scratch\analise-dre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14FB826C-3122-4368-9A26-D94C0D47D88A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DF744CD-C47E-46B2-977E-84C94F8F53F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="706" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="706" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Indicadores" sheetId="10" state="hidden" r:id="rId1"/>
@@ -739,7 +739,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -950,12 +950,11 @@
     <xf numFmtId="16" fontId="5" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -1349,17 +1348,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BCC6A2B-3058-4004-816D-7182CED8014F}">
   <dimension ref="A1:I134"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.109375" customWidth="1"/>
+    <col min="1" max="1" width="22.140625" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="37" customWidth="1"/>
-    <col min="7" max="7" width="14.109375" customWidth="1"/>
-    <col min="8" max="8" width="11.5546875" customWidth="1"/>
+    <col min="7" max="7" width="14.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -1379,7 +1378,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1400,7 +1399,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1421,7 +1420,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1442,7 +1441,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1463,7 +1462,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1484,7 +1483,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1505,7 +1504,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1526,7 +1525,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1547,7 +1546,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1568,7 +1567,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -1589,7 +1588,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1610,7 +1609,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -1631,7 +1630,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -1652,7 +1651,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -1673,7 +1672,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>4</v>
       </c>
@@ -1694,7 +1693,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>4</v>
       </c>
@@ -1715,7 +1714,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>4</v>
       </c>
@@ -1736,7 +1735,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>4</v>
       </c>
@@ -1757,7 +1756,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>4</v>
       </c>
@@ -1778,7 +1777,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>4</v>
       </c>
@@ -1799,7 +1798,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>4</v>
       </c>
@@ -1820,7 +1819,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>4</v>
       </c>
@@ -1841,7 +1840,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>4</v>
       </c>
@@ -1862,7 +1861,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>4</v>
       </c>
@@ -1883,7 +1882,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>4</v>
       </c>
@@ -1902,7 +1901,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>4</v>
       </c>
@@ -1921,7 +1920,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>4</v>
       </c>
@@ -1940,7 +1939,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>4</v>
       </c>
@@ -1959,7 +1958,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>4</v>
       </c>
@@ -1978,7 +1977,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>4</v>
       </c>
@@ -1997,7 +1996,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>4</v>
       </c>
@@ -2016,7 +2015,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>4</v>
       </c>
@@ -2035,7 +2034,7 @@
         <v>HALL DESIGN Margem</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>4</v>
       </c>
@@ -2056,7 +2055,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>4</v>
       </c>
@@ -2077,7 +2076,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>4</v>
       </c>
@@ -2098,7 +2097,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>4</v>
       </c>
@@ -2119,7 +2118,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>4</v>
       </c>
@@ -2140,7 +2139,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>4</v>
       </c>
@@ -2161,7 +2160,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>4</v>
       </c>
@@ -2182,7 +2181,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>4</v>
       </c>
@@ -2203,7 +2202,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>4</v>
       </c>
@@ -2224,7 +2223,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>4</v>
       </c>
@@ -2245,7 +2244,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>4</v>
       </c>
@@ -2266,7 +2265,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>4</v>
       </c>
@@ -2287,7 +2286,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>4</v>
       </c>
@@ -2308,7 +2307,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>4</v>
       </c>
@@ -2329,7 +2328,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>4</v>
       </c>
@@ -2350,7 +2349,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>4</v>
       </c>
@@ -2371,7 +2370,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>4</v>
       </c>
@@ -2392,7 +2391,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>4</v>
       </c>
@@ -2413,7 +2412,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>4</v>
       </c>
@@ -2434,7 +2433,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>4</v>
       </c>
@@ -2455,7 +2454,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>4</v>
       </c>
@@ -2476,7 +2475,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>4</v>
       </c>
@@ -2497,7 +2496,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>4</v>
       </c>
@@ -2518,7 +2517,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>4</v>
       </c>
@@ -2539,7 +2538,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>4</v>
       </c>
@@ -2558,7 +2557,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>4</v>
       </c>
@@ -2577,7 +2576,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>4</v>
       </c>
@@ -2596,7 +2595,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>4</v>
       </c>
@@ -2615,7 +2614,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>4</v>
       </c>
@@ -2634,7 +2633,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>4</v>
       </c>
@@ -2653,7 +2652,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>4</v>
       </c>
@@ -2672,7 +2671,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>4</v>
       </c>
@@ -2691,7 +2690,7 @@
         <v>HALL DESIGN Resultado</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>4</v>
       </c>
@@ -2719,7 +2718,7 @@
         <v>2.5976243171854298E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>4</v>
       </c>
@@ -2747,7 +2746,7 @@
         <v>4.4489038312087614E-2</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>4</v>
       </c>
@@ -2775,7 +2774,7 @@
         <v>4.9493272643934147E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>4</v>
       </c>
@@ -2803,7 +2802,7 @@
         <v>4.9113724641000805E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>4</v>
       </c>
@@ -2834,7 +2833,7 @@
         <v>6.3615727856344131E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>4</v>
       </c>
@@ -2855,7 +2854,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>4</v>
       </c>
@@ -2876,7 +2875,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>4</v>
       </c>
@@ -2897,7 +2896,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>4</v>
       </c>
@@ -2918,7 +2917,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>4</v>
       </c>
@@ -2937,7 +2936,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>4</v>
       </c>
@@ -2956,7 +2955,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>4</v>
       </c>
@@ -2975,7 +2974,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>4</v>
       </c>
@@ -2994,7 +2993,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>4</v>
       </c>
@@ -3013,7 +3012,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>4</v>
       </c>
@@ -3032,7 +3031,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>4</v>
       </c>
@@ -3051,7 +3050,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>4</v>
       </c>
@@ -3070,7 +3069,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>4</v>
       </c>
@@ -3089,7 +3088,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>4</v>
       </c>
@@ -3108,7 +3107,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>4</v>
       </c>
@@ -3127,7 +3126,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>4</v>
       </c>
@@ -3146,7 +3145,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>4</v>
       </c>
@@ -3165,7 +3164,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>4</v>
       </c>
@@ -3184,7 +3183,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>4</v>
       </c>
@@ -3203,7 +3202,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>4</v>
       </c>
@@ -3223,7 +3222,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>4</v>
       </c>
@@ -3243,7 +3242,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>4</v>
       </c>
@@ -3263,7 +3262,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>4</v>
       </c>
@@ -3283,7 +3282,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>4</v>
       </c>
@@ -3303,7 +3302,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>4</v>
       </c>
@@ -3323,7 +3322,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>4</v>
       </c>
@@ -3343,7 +3342,7 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>4</v>
       </c>
@@ -3363,8 +3362,8 @@
         <v>HALL DESIGN Despesas ADM</v>
       </c>
     </row>
-    <row r="101" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>4</v>
       </c>
@@ -3383,7 +3382,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>4</v>
       </c>
@@ -3402,7 +3401,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>4</v>
       </c>
@@ -3421,7 +3420,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>4</v>
       </c>
@@ -3440,7 +3439,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>4</v>
       </c>
@@ -3459,7 +3458,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>4</v>
       </c>
@@ -3478,7 +3477,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>4</v>
       </c>
@@ -3497,7 +3496,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>4</v>
       </c>
@@ -3516,7 +3515,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>4</v>
       </c>
@@ -3535,7 +3534,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>4</v>
       </c>
@@ -3554,7 +3553,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>4</v>
       </c>
@@ -3573,7 +3572,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>4</v>
       </c>
@@ -3592,7 +3591,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>4</v>
       </c>
@@ -3611,7 +3610,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>4</v>
       </c>
@@ -3630,7 +3629,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>4</v>
       </c>
@@ -3649,7 +3648,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>4</v>
       </c>
@@ -3668,7 +3667,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>4</v>
       </c>
@@ -3687,7 +3686,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>4</v>
       </c>
@@ -3706,7 +3705,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>4</v>
       </c>
@@ -3725,7 +3724,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>4</v>
       </c>
@@ -3744,7 +3743,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>4</v>
       </c>
@@ -3763,7 +3762,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>4</v>
       </c>
@@ -3782,7 +3781,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>4</v>
       </c>
@@ -3801,7 +3800,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>4</v>
       </c>
@@ -3820,7 +3819,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>4</v>
       </c>
@@ -3840,7 +3839,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>4</v>
       </c>
@@ -3860,7 +3859,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>4</v>
       </c>
@@ -3880,7 +3879,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>4</v>
       </c>
@@ -3900,7 +3899,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>4</v>
       </c>
@@ -3920,7 +3919,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>4</v>
       </c>
@@ -3940,7 +3939,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>4</v>
       </c>
@@ -3960,7 +3959,7 @@
         <v>HALL DESIGN % Receita liquida geral</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>4</v>
       </c>
@@ -3989,26 +3988,26 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3B648EA-C9CF-4199-AC21-3B599FE2C0B5}">
   <sheetPr codeName="Planilha4"/>
   <dimension ref="A1:S25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="15.5546875" customWidth="1"/>
-    <col min="5" max="5" width="20.109375" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="5" max="5" width="20.140625" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="15.5546875" customWidth="1"/>
+    <col min="7" max="7" width="15.5703125" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="12" width="15.5546875" customWidth="1"/>
-    <col min="13" max="13" width="25.88671875" customWidth="1"/>
+    <col min="9" max="12" width="15.5703125" customWidth="1"/>
+    <col min="13" max="13" width="25.85546875" customWidth="1"/>
     <col min="14" max="14" width="15" customWidth="1"/>
-    <col min="15" max="15" width="42.88671875" customWidth="1"/>
-    <col min="16" max="16" width="15.88671875" customWidth="1"/>
-    <col min="17" max="17" width="15.44140625" customWidth="1"/>
-    <col min="18" max="18" width="21.33203125" customWidth="1"/>
+    <col min="15" max="15" width="42.85546875" customWidth="1"/>
+    <col min="16" max="16" width="15.85546875" customWidth="1"/>
+    <col min="17" max="17" width="15.42578125" customWidth="1"/>
+    <col min="18" max="18" width="21.28515625" customWidth="1"/>
     <col min="19" max="19" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:19" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -4067,7 +4066,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="45" t="s">
         <v>14</v>
       </c>
@@ -4129,7 +4128,7 @@
         <v>4.9500000000000002E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="46" t="s">
         <v>57</v>
       </c>
@@ -4192,7 +4191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="47" t="s">
         <v>16</v>
       </c>
@@ -4231,7 +4230,7 @@
         <v>24</v>
       </c>
       <c r="L4" s="31">
-        <f t="shared" ref="L3:L25" si="4">K4*J4</f>
+        <f t="shared" ref="L4:L25" si="4">K4*J4</f>
         <v>1382966.16</v>
       </c>
       <c r="M4" s="35"/>
@@ -4255,7 +4254,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="47" t="s">
         <v>76</v>
       </c>
@@ -4317,7 +4316,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="47" t="s">
         <v>77</v>
       </c>
@@ -4379,7 +4378,7 @@
         <v>3.9599999999999996E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="47" t="s">
         <v>20</v>
       </c>
@@ -4442,7 +4441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="47" t="s">
         <v>22</v>
       </c>
@@ -4505,7 +4504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="47" t="s">
         <v>23</v>
       </c>
@@ -4569,7 +4568,7 @@
         <v>1.9799999999999998E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="47" t="s">
         <v>24</v>
       </c>
@@ -4632,7 +4631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="47" t="s">
         <v>25</v>
       </c>
@@ -4696,7 +4695,7 @@
         <v>4.9500000000000002E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="47" t="s">
         <v>26</v>
       </c>
@@ -4760,7 +4759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="47" t="s">
         <v>27</v>
       </c>
@@ -4822,7 +4821,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="47" t="s">
         <v>28</v>
       </c>
@@ -4884,7 +4883,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="47" t="s">
         <v>29</v>
       </c>
@@ -4946,7 +4945,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="47" t="s">
         <v>30</v>
       </c>
@@ -5008,7 +5007,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="47" t="s">
         <v>31</v>
       </c>
@@ -5070,7 +5069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="47" t="s">
         <v>32</v>
       </c>
@@ -5132,7 +5131,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="47" t="s">
         <v>33</v>
       </c>
@@ -5194,7 +5193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="47" t="s">
         <v>61</v>
       </c>
@@ -5256,7 +5255,7 @@
         <v>1.9799999999999998E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="48" t="s">
         <v>62</v>
       </c>
@@ -5317,7 +5316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="63" t="s">
         <v>80</v>
       </c>
@@ -5374,7 +5373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="63" t="s">
         <v>63</v>
       </c>
@@ -5434,7 +5433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="63" t="s">
         <v>79</v>
       </c>
@@ -5494,7 +5493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A25" s="63" t="s">
         <v>78</v>
       </c>
@@ -5535,7 +5534,7 @@
       <c r="N25" s="75" t="s">
         <v>84</v>
       </c>
-      <c r="O25" s="79" t="s">
+      <c r="O25" t="s">
         <v>96</v>
       </c>
       <c r="P25" s="28">
@@ -5544,7 +5543,7 @@
       <c r="Q25" s="65">
         <v>22244837</v>
       </c>
-      <c r="R25" s="80">
+      <c r="R25" s="8">
         <f>IF(I25&gt;0,Q25*P25,0)</f>
         <v>0</v>
       </c>
@@ -5562,19 +5561,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9847408C-B23C-4D48-83D1-CB6301E525D5}">
   <sheetPr codeName="Planilha5"/>
-  <dimension ref="A1:M26"/>
-  <sheetFormatPr defaultRowHeight="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:M29"/>
+  <sheetFormatPr defaultRowHeight="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="36.44140625" customWidth="1"/>
-    <col min="3" max="8" width="27.88671875" customWidth="1"/>
-    <col min="9" max="9" width="36.44140625" style="62" customWidth="1"/>
-    <col min="10" max="10" width="36.44140625" customWidth="1"/>
-    <col min="11" max="11" width="24.5546875" customWidth="1"/>
+    <col min="1" max="2" width="36.42578125" customWidth="1"/>
+    <col min="3" max="8" width="27.85546875" customWidth="1"/>
+    <col min="9" max="9" width="36.42578125" style="62" customWidth="1"/>
+    <col min="10" max="10" width="36.42578125" customWidth="1"/>
+    <col min="11" max="11" width="24.5703125" customWidth="1"/>
     <col min="12" max="12" width="26" customWidth="1"/>
-    <col min="13" max="13" width="255.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="255.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -5615,7 +5614,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="45" t="s">
         <v>14</v>
       </c>
@@ -5645,7 +5644,10 @@
         <v>-5230293.6999999955</v>
       </c>
       <c r="I2" s="60"/>
-      <c r="J2" s="20"/>
+      <c r="J2" s="79">
+        <f>H2</f>
+        <v>-5230293.6999999955</v>
+      </c>
       <c r="K2" s="20"/>
       <c r="L2" s="24">
         <v>0</v>
@@ -5654,7 +5656,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="46" t="s">
         <v>57</v>
       </c>
@@ -5690,7 +5692,7 @@
       <c r="L3" s="24"/>
       <c r="M3" s="44"/>
     </row>
-    <row r="4" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="47" t="s">
         <v>16</v>
       </c>
@@ -5727,7 +5729,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="47" t="s">
         <v>4</v>
       </c>
@@ -5770,7 +5772,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="47" t="s">
         <v>3</v>
       </c>
@@ -5809,7 +5811,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="47" t="s">
         <v>20</v>
       </c>
@@ -5846,7 +5848,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="47" t="s">
         <v>22</v>
       </c>
@@ -5883,7 +5885,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="47" t="s">
         <v>23</v>
       </c>
@@ -5926,7 +5928,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="47" t="s">
         <v>24</v>
       </c>
@@ -5966,7 +5968,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="47" t="s">
         <v>25</v>
       </c>
@@ -6009,7 +6011,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="47" t="s">
         <v>26</v>
       </c>
@@ -6049,7 +6051,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="47" t="s">
         <v>27</v>
       </c>
@@ -6089,7 +6091,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="47" t="s">
         <v>28</v>
       </c>
@@ -6129,7 +6131,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="47" t="s">
         <v>29</v>
       </c>
@@ -6169,7 +6171,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="47" t="s">
         <v>30</v>
       </c>
@@ -6209,7 +6211,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="47" t="s">
         <v>31</v>
       </c>
@@ -6249,7 +6251,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="47" t="s">
         <v>32</v>
       </c>
@@ -6289,7 +6291,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="47" t="s">
         <v>33</v>
       </c>
@@ -6329,7 +6331,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="47" t="s">
         <v>61</v>
       </c>
@@ -6369,7 +6371,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="48" t="s">
         <v>62</v>
       </c>
@@ -6409,7 +6411,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="63" t="s">
         <v>67</v>
       </c>
@@ -6449,7 +6451,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="63" t="s">
         <v>63</v>
       </c>
@@ -6487,7 +6489,7 @@
       </c>
       <c r="M23" s="68"/>
     </row>
-    <row r="24" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="63" t="s">
         <v>64</v>
       </c>
@@ -6529,7 +6531,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="63" t="s">
         <v>65</v>
       </c>
@@ -6559,8 +6561,14 @@
         <v>-83239</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D26" s="59"/>
+    </row>
+    <row r="29" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J29">
+        <f>K15</f>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:L21" xr:uid="{F826C8AD-E55D-43EC-8E13-5835E0D42917}"/>

</xml_diff>